<commit_message>
Start looking at Naigles data
</commit_message>
<xml_diff>
--- a/data/CDI_asd.xlsx
+++ b/data/CDI_asd.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/teclis/Desktop/PAPERS/ADJ/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\swest19\Desktop\Check-ASD-Subs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FBB7F82-8C5C-8843-9A88-E8FDBCAD1DCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A3CBD29-045A-40A2-86DF-E917DF520B8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9520" yWindow="1240" windowWidth="27240" windowHeight="16440" xr2:uid="{B98226F3-B36F-2746-A52C-A26C5CA0EDCD}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{B98226F3-B36F-2746-A52C-A26C5CA0EDCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,14 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>ID</t>
   </si>
   <si>
-    <t>V1_W_G_says</t>
-  </si>
-  <si>
     <t>ASD_2_a</t>
   </si>
   <si>
@@ -140,58 +137,28 @@
     <t>ASD_3_o</t>
   </si>
   <si>
-    <t>C1_1</t>
-  </si>
-  <si>
-    <t>C1_2</t>
-  </si>
-  <si>
-    <t>C1_3</t>
-  </si>
-  <si>
-    <t>C1_4</t>
-  </si>
-  <si>
-    <t>C1_5</t>
-  </si>
-  <si>
-    <t>C1_6</t>
-  </si>
-  <si>
-    <t>C1_7</t>
-  </si>
-  <si>
-    <t>C1_8</t>
-  </si>
-  <si>
-    <t>C1_9</t>
-  </si>
-  <si>
-    <t>C1_10</t>
-  </si>
-  <si>
     <t>V2_age</t>
   </si>
   <si>
-    <t>V2_W_G_says</t>
-  </si>
-  <si>
-    <t>V2CDITotalwords_W_P</t>
-  </si>
-  <si>
-    <t>V3Age</t>
-  </si>
-  <si>
-    <t>V3CDITotalwords_WP</t>
-  </si>
-  <si>
-    <t>V1_Age</t>
-  </si>
-  <si>
     <t>INFANT</t>
   </si>
   <si>
     <t>TODDLER</t>
+  </si>
+  <si>
+    <t>V1_produced</t>
+  </si>
+  <si>
+    <t>V1_age</t>
+  </si>
+  <si>
+    <t>V2_produced</t>
+  </si>
+  <si>
+    <t>V3_age</t>
+  </si>
+  <si>
+    <t>V3_produced</t>
   </si>
 </sst>
 </file>
@@ -258,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -267,10 +234,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -605,55 +571,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD3F009A-B87A-A840-967E-93CE66EF705C}">
-  <dimension ref="A1:I44"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:H44"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="2"/>
+    <col min="1" max="1" width="10.875" style="2"/>
+    <col min="3" max="3" width="14.5" customWidth="1"/>
+    <col min="5" max="5" width="28.625" customWidth="1"/>
+    <col min="6" max="6" width="19.375" customWidth="1"/>
+    <col min="7" max="7" width="20.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B1" s="4" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="5" t="s">
-        <v>51</v>
-      </c>
+      <c r="E1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F1" s="5"/>
       <c r="G1" s="5"/>
       <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F2" t="s">
-        <v>46</v>
-      </c>
-      <c r="G2" t="s">
-        <v>47</v>
-      </c>
-      <c r="H2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
-        <v>2</v>
       </c>
       <c r="B3">
         <v>29.47</v>
@@ -664,19 +630,19 @@
       <c r="D3">
         <v>33.232999999999997</v>
       </c>
+      <c r="E3">
+        <v>549</v>
+      </c>
       <c r="F3">
-        <v>549</v>
+        <v>37.33</v>
       </c>
       <c r="G3">
-        <v>37.33</v>
-      </c>
-      <c r="H3">
         <v>569</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4">
         <v>31.17</v>
@@ -687,19 +653,19 @@
       <c r="D4">
         <v>35.299999999999997</v>
       </c>
+      <c r="E4">
+        <v>480</v>
+      </c>
       <c r="F4">
-        <v>480</v>
+        <v>38.9</v>
       </c>
       <c r="G4">
-        <v>38.9</v>
-      </c>
-      <c r="H4">
         <v>461</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5">
         <v>34.229999999999997</v>
@@ -710,19 +676,19 @@
       <c r="D5">
         <v>37.700000000000003</v>
       </c>
+      <c r="E5">
+        <v>387</v>
+      </c>
       <c r="F5">
-        <v>387</v>
+        <v>41.63</v>
       </c>
       <c r="G5">
-        <v>41.63</v>
-      </c>
-      <c r="H5">
         <v>577</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="3">
         <v>30.1</v>
@@ -733,20 +699,19 @@
       <c r="D6" s="3">
         <v>33.799999999999997</v>
       </c>
-      <c r="E6" s="3"/>
+      <c r="E6" s="3">
+        <v>218</v>
+      </c>
       <c r="F6" s="3">
-        <v>218</v>
+        <v>37.43</v>
       </c>
       <c r="G6" s="3">
-        <v>37.43</v>
-      </c>
-      <c r="H6" s="3">
         <v>253</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7">
         <v>28.1</v>
@@ -757,19 +722,19 @@
       <c r="D7">
         <v>33.5</v>
       </c>
+      <c r="E7">
+        <v>650</v>
+      </c>
       <c r="F7">
-        <v>650</v>
+        <v>36.229999999999997</v>
       </c>
       <c r="G7">
-        <v>36.229999999999997</v>
-      </c>
-      <c r="H7">
         <v>563</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="3">
         <v>34.83</v>
@@ -780,14 +745,13 @@
       <c r="D8" s="3">
         <v>38.729999999999997</v>
       </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3">
+      <c r="E8" s="3">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9">
         <v>35.83</v>
@@ -798,19 +762,19 @@
       <c r="D9">
         <v>39.93</v>
       </c>
+      <c r="E9">
+        <v>228</v>
+      </c>
       <c r="F9">
-        <v>228</v>
+        <v>43.9</v>
       </c>
       <c r="G9">
-        <v>43.9</v>
-      </c>
-      <c r="H9">
         <v>326</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="3">
         <v>37.53</v>
@@ -821,20 +785,19 @@
       <c r="D10" s="3">
         <v>42.2</v>
       </c>
-      <c r="E10" s="3"/>
+      <c r="E10" s="3">
+        <v>19</v>
+      </c>
       <c r="F10" s="3">
-        <v>19</v>
+        <v>46.37</v>
       </c>
       <c r="G10" s="3">
-        <v>46.37</v>
-      </c>
-      <c r="H10" s="3">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11">
         <v>30.93</v>
@@ -845,19 +808,19 @@
       <c r="D11">
         <v>34.67</v>
       </c>
+      <c r="E11">
+        <v>432</v>
+      </c>
       <c r="F11">
-        <v>432</v>
+        <v>38.770000000000003</v>
       </c>
       <c r="G11">
-        <v>38.770000000000003</v>
-      </c>
-      <c r="H11">
         <v>580</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12">
         <v>34.47</v>
@@ -868,19 +831,19 @@
       <c r="D12">
         <v>38.57</v>
       </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
       <c r="F12">
-        <v>0</v>
+        <v>42.2</v>
       </c>
       <c r="G12">
-        <v>42.2</v>
-      </c>
-      <c r="H12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="3">
         <v>34</v>
@@ -891,20 +854,19 @@
       <c r="D13" s="3">
         <v>38.130000000000003</v>
       </c>
-      <c r="E13" s="3"/>
+      <c r="E13" s="3">
+        <v>370</v>
+      </c>
       <c r="F13" s="3">
-        <v>370</v>
+        <v>42.27</v>
       </c>
       <c r="G13" s="3">
-        <v>42.27</v>
-      </c>
-      <c r="H13" s="3">
         <v>423</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" s="3">
         <v>33.4</v>
@@ -915,20 +877,19 @@
       <c r="D14" s="3">
         <v>37.4</v>
       </c>
-      <c r="E14" s="3"/>
+      <c r="E14" s="3">
+        <v>154</v>
+      </c>
       <c r="F14" s="3">
-        <v>154</v>
+        <v>41.77</v>
       </c>
       <c r="G14" s="3">
-        <v>41.77</v>
-      </c>
-      <c r="H14" s="3">
         <v>135</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15">
         <v>37.200000000000003</v>
@@ -939,19 +900,19 @@
       <c r="D15">
         <v>41.53</v>
       </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
       <c r="F15">
-        <v>0</v>
+        <v>45.57</v>
       </c>
       <c r="G15">
-        <v>45.57</v>
-      </c>
-      <c r="H15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16">
         <v>31.8</v>
@@ -962,13 +923,13 @@
       <c r="D16">
         <v>36.67</v>
       </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17">
         <v>37.869999999999997</v>
@@ -979,19 +940,19 @@
       <c r="D17">
         <v>42.2</v>
       </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
       <c r="F17">
-        <v>3</v>
+        <v>46.37</v>
       </c>
       <c r="G17">
-        <v>46.37</v>
-      </c>
-      <c r="H17">
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18">
         <v>35.53</v>
@@ -1002,19 +963,19 @@
       <c r="D18">
         <v>39.4</v>
       </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
       <c r="F18">
-        <v>1</v>
+        <v>44.47</v>
       </c>
       <c r="G18">
-        <v>44.47</v>
-      </c>
-      <c r="H18">
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" s="3">
         <v>26.17</v>
@@ -1025,20 +986,19 @@
       <c r="D19" s="3">
         <v>30.3</v>
       </c>
-      <c r="E19" s="3"/>
+      <c r="E19" s="3">
+        <v>219</v>
+      </c>
       <c r="F19" s="3">
-        <v>219</v>
+        <v>34.229999999999997</v>
       </c>
       <c r="G19" s="3">
-        <v>34.229999999999997</v>
-      </c>
-      <c r="H19" s="3">
         <v>330</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="3">
         <v>26.17</v>
@@ -1049,20 +1009,19 @@
       <c r="D20" s="3">
         <v>30.27</v>
       </c>
-      <c r="E20" s="3"/>
+      <c r="E20" s="3">
+        <v>56</v>
+      </c>
       <c r="F20" s="3">
-        <v>56</v>
+        <v>34.57</v>
       </c>
       <c r="G20" s="3">
-        <v>34.57</v>
-      </c>
-      <c r="H20" s="3">
         <v>242</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21">
         <v>41</v>
@@ -1073,19 +1032,19 @@
       <c r="D21">
         <v>44.6</v>
       </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
       <c r="F21">
-        <v>0</v>
+        <v>49.2</v>
       </c>
       <c r="G21">
-        <v>49.2</v>
-      </c>
-      <c r="H21">
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22">
         <v>32.369999999999997</v>
@@ -1096,19 +1055,19 @@
       <c r="D22">
         <v>30.5</v>
       </c>
+      <c r="E22">
+        <v>12</v>
+      </c>
       <c r="F22">
-        <v>12</v>
+        <v>40.130000000000003</v>
       </c>
       <c r="G22">
-        <v>40.130000000000003</v>
-      </c>
-      <c r="H22">
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" s="3">
         <v>18.77</v>
@@ -1119,20 +1078,19 @@
       <c r="D23" s="3">
         <v>22.5</v>
       </c>
-      <c r="E23" s="3"/>
+      <c r="E23" s="3">
+        <v>138</v>
+      </c>
       <c r="F23" s="3">
-        <v>138</v>
+        <v>26.77</v>
       </c>
       <c r="G23" s="3">
-        <v>26.77</v>
-      </c>
-      <c r="H23" s="3">
         <v>288</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24">
         <v>27.53</v>
@@ -1140,16 +1098,16 @@
       <c r="C24">
         <v>1</v>
       </c>
+      <c r="F24">
+        <v>36.17</v>
+      </c>
       <c r="G24">
-        <v>36.17</v>
-      </c>
-      <c r="H24">
         <v>148</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" s="3">
         <v>27.37</v>
@@ -1160,20 +1118,19 @@
       <c r="D25" s="3">
         <v>32.1</v>
       </c>
-      <c r="E25" s="3"/>
+      <c r="E25" s="3">
+        <v>135</v>
+      </c>
       <c r="F25" s="3">
-        <v>135</v>
+        <v>35.6</v>
       </c>
       <c r="G25" s="3">
-        <v>35.6</v>
-      </c>
-      <c r="H25" s="3">
         <v>193</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B26" s="3">
         <v>34.869999999999997</v>
@@ -1184,20 +1141,19 @@
       <c r="D26" s="3">
         <v>38.130000000000003</v>
       </c>
-      <c r="E26" s="3"/>
+      <c r="E26" s="3">
+        <v>105</v>
+      </c>
       <c r="F26" s="3">
-        <v>105</v>
+        <v>43.1</v>
       </c>
       <c r="G26" s="3">
-        <v>43.1</v>
-      </c>
-      <c r="H26" s="3">
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" s="3">
         <v>36.53</v>
@@ -1208,20 +1164,19 @@
       <c r="D27" s="3">
         <v>40.630000000000003</v>
       </c>
-      <c r="E27" s="3"/>
+      <c r="E27" s="3">
+        <v>19</v>
+      </c>
       <c r="F27" s="3">
-        <v>19</v>
+        <v>44.67</v>
       </c>
       <c r="G27" s="3">
-        <v>44.67</v>
-      </c>
-      <c r="H27" s="3">
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28">
         <v>25.33</v>
@@ -1232,19 +1187,19 @@
       <c r="D28">
         <v>29.7</v>
       </c>
+      <c r="E28">
+        <v>3</v>
+      </c>
       <c r="F28">
-        <v>3</v>
+        <v>34.1</v>
       </c>
       <c r="G28">
-        <v>34.1</v>
-      </c>
-      <c r="H28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" s="3">
         <v>39.5</v>
@@ -1255,20 +1210,19 @@
       <c r="D29" s="3">
         <v>43.68</v>
       </c>
-      <c r="E29" s="3"/>
+      <c r="E29" s="3">
+        <v>449</v>
+      </c>
       <c r="F29" s="3">
-        <v>449</v>
+        <v>47.73</v>
       </c>
       <c r="G29" s="3">
-        <v>47.73</v>
-      </c>
-      <c r="H29" s="3">
         <v>390</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30">
         <v>24.9</v>
@@ -1279,13 +1233,13 @@
       <c r="D30">
         <v>32.200000000000003</v>
       </c>
-      <c r="F30">
+      <c r="E30">
         <v>121</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31">
         <v>37.03</v>
@@ -1296,13 +1250,13 @@
       <c r="D31">
         <v>42.77</v>
       </c>
-      <c r="F31">
+      <c r="E31">
         <v>670</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B32">
         <v>41.07</v>
@@ -1313,19 +1267,19 @@
       <c r="D32">
         <v>41.07</v>
       </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
       <c r="F32">
-        <v>0</v>
+        <v>49.97</v>
       </c>
       <c r="G32">
-        <v>49.97</v>
-      </c>
-      <c r="H32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33">
         <v>34</v>
@@ -1336,19 +1290,19 @@
       <c r="D33">
         <v>38.630000000000003</v>
       </c>
+      <c r="E33">
+        <v>456</v>
+      </c>
       <c r="F33">
-        <v>456</v>
+        <v>42.47</v>
       </c>
       <c r="G33">
-        <v>42.47</v>
-      </c>
-      <c r="H33">
         <v>467</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" s="3">
         <v>42</v>
@@ -1359,154 +1313,65 @@
       <c r="D34" s="3">
         <v>46.77</v>
       </c>
-      <c r="E34" s="3"/>
+      <c r="E34" s="3">
+        <v>201</v>
+      </c>
       <c r="F34" s="3">
-        <v>201</v>
+        <v>50.63</v>
       </c>
       <c r="G34" s="3">
-        <v>50.63</v>
-      </c>
-      <c r="H34" s="3">
         <v>392</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="C35" s="1">
-        <v>36</v>
-      </c>
-      <c r="D35" s="1">
-        <v>45</v>
-      </c>
-      <c r="E35" s="1">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C36" s="1">
-        <v>7</v>
-      </c>
-      <c r="D36" s="1">
-        <v>36</v>
-      </c>
-      <c r="E36" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C37" s="1">
-        <v>155</v>
-      </c>
-      <c r="D37" s="1">
-        <v>34.5</v>
-      </c>
-      <c r="E37" s="1">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A38" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C38" s="1">
-        <v>86</v>
-      </c>
-      <c r="D38" s="1">
-        <v>32</v>
-      </c>
-      <c r="E38" s="1">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A39" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C39" s="1">
-        <v>22</v>
-      </c>
-      <c r="D39" s="1">
-        <v>37</v>
-      </c>
-      <c r="E39" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C40" s="1">
-        <v>43</v>
-      </c>
-      <c r="D40" s="1">
-        <v>35</v>
-      </c>
-      <c r="E40" s="1"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C41" s="1">
-        <v>177</v>
-      </c>
-      <c r="D41" s="1">
-        <v>42</v>
-      </c>
-      <c r="E41" s="1">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="C42" s="1">
-        <v>40</v>
-      </c>
-      <c r="D42" s="1">
-        <v>35</v>
-      </c>
-      <c r="E42" s="1">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C43" s="1">
-        <v>217</v>
-      </c>
-      <c r="D43" s="1">
-        <v>44</v>
-      </c>
-      <c r="E43" s="1">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A44" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C44" s="1">
-        <v>137</v>
-      </c>
-      <c r="D44" s="1">
-        <v>40.5</v>
-      </c>
-      <c r="E44" s="1">
-        <v>281</v>
-      </c>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="1"/>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="1"/>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="1"/>
+      <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="1"/>
+      <c r="C41" s="1"/>
+      <c r="D41" s="1"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="1"/>
+      <c r="C42" s="1"/>
+      <c r="D42" s="1"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="1"/>
+      <c r="C43" s="1"/>
+      <c r="D43" s="1"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="1"/>
+      <c r="C44" s="1"/>
+      <c r="D44" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>